<commit_message>
[2D Game Project] 일단 Stage화면 전까지 로드 완료
</commit_message>
<xml_diff>
--- a/ExcelFiles/character.xlsx
+++ b/ExcelFiles/character.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OzProject\UnityBasic_6\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OzProject\UnityProject\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F361B6-5AC3-4640-AE1C-9CC53C66E873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343E54B3-5471-4200-851A-793B080CDAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F95A0D0-2173-408D-8AC8-2EE339C7D472}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>character_punch_01</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -88,6 +88,62 @@
   </si>
   <si>
     <t>Card</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Animator/punch_controller</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Animator/gun_controller</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Animator/knife_controller</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharacterAnimAddress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharacterImageAddress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharacterImageSpriteName</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/punch_idle</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/gun_idle</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/knife_idle</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>punch_idle_0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>knife_idle_0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gun_idle_0</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -452,21 +508,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98541795-7E49-4832-8414-4CA1CDD3C226}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="31.296875" customWidth="1"/>
     <col min="2" max="2" width="38.09765625" customWidth="1"/>
     <col min="3" max="3" width="31.796875" customWidth="1"/>
     <col min="4" max="4" width="32.19921875" customWidth="1"/>
+    <col min="5" max="5" width="43.3984375" customWidth="1"/>
+    <col min="6" max="6" width="30.796875" customWidth="1"/>
+    <col min="7" max="7" width="27.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -476,8 +535,20 @@
       <c r="C2" t="s">
         <v>12</v>
       </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -487,8 +558,20 @@
       <c r="C3" t="s">
         <v>15</v>
       </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -498,8 +581,20 @@
       <c r="C4" t="s">
         <v>6</v>
       </c>
+      <c r="D4">
+        <v>70</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -509,8 +604,20 @@
       <c r="C5" t="s">
         <v>7</v>
       </c>
+      <c r="D5">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -519,6 +626,18 @@
       </c>
       <c r="C6" t="s">
         <v>8</v>
+      </c>
+      <c r="D6">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>